<commit_message>
2025 08 17 Chapter 1 Working Session
</commit_message>
<xml_diff>
--- a/Lessons_and_Logs/Neural_Networks/Chapter_1/Notes/Chapter_1_Data.xlsx
+++ b/Lessons_and_Logs/Neural_Networks/Chapter_1/Notes/Chapter_1_Data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/99d2d0efc5e421e1/Working_Files/Code/Repositories/Python/Lessons_and_Logs/Neural_Networks/Chapter_1/Notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37D5DFB8-738E-4363-8432-B41E266474C1}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="11_F25DC773A252ABDACC1048B0395B70645BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C047C04-7FA9-4FCC-A773-EB3B9DF05234}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="30 Epochs 30 Hidden Nodes" sheetId="1" r:id="rId1"/>
+    <sheet name="30 Epochs 30 Hidden Neurons" sheetId="1" r:id="rId1"/>
+    <sheet name="30 Epochs 100 Hidden Neurons" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="443">
   <si>
     <t>Epoch 0: 9095 / 10000</t>
   </si>
@@ -681,6 +682,690 @@
   </si>
   <si>
     <t>Epoch 29: 9504 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 0: 9003 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 9213 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 2: 9307 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 9359 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 9364 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 5: 9420 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 9381 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 7: 9423 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 9437 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 9420 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 10: 9435 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 9451 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 13: 9449 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 9461 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 9463 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 9480 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 9475 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 18: 9476 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 9461 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 9486 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 9482 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 23: 9500 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 9480 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 9453 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 26: 9499 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 9519 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 28: 9514 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 9473 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 0: 7918 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 9184 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 9324 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 9378 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 5: 9394 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 9390 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 9412 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 9421 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 9452 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 12: 9455 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 13: 9479 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 9463 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 9473 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 9499 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 9499 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 18: 9492 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 9507 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 9505 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 9501 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 22: 9507 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 23: 9505 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 9523 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 9491 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 26: 9467 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 9475 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 9534 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 0: 9057 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 9228 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 2: 9290 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 9365 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 9359 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 9369 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 7: 9426 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 9414 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 9418 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 9466 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 12: 9428 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 9480 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 9480 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 9461 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 9482 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 18: 9506 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 9487 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 9492 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 9462 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 22: 9496 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 9530 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 9504 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 26: 9496 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 9513 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 28: 9517 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 9512 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 0: 9090 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 9236 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 2: 9322 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 9381 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 9409 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 9427 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 7: 9427 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 9441 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 9458 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 10: 9450 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 9465 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 13: 9478 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 9479 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 9498 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 9479 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 9472 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 9498 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 9484 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 9485 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 22: 9495 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 23: 9473 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 9484 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 9466 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 9502 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 28: 9494 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 9495 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 0: 7419 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 7543 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 2: 7632 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 7664 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 7683 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 5: 7690 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 7711 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 7: 7705 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 7717 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 7738 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 10: 7730 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 7730 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 12: 7743 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 13: 7740 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 7753 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 7742 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 7766 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 7762 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 18: 7763 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 7764 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 7766 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 7771 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 22: 7776 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 23: 7775 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 7785 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 7783 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 26: 7786 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 7781 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 28: 7784 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 7787 / 10000</t>
+  </si>
+  <si>
+    <t>net.SGD(training_data, 30, 10, 3.0, test_data=test_data)</t>
+  </si>
+  <si>
+    <t>net.SGD(training_data, 30, 10, 6.0, test_data=test_data)</t>
+  </si>
+  <si>
+    <t>Epoch 0: 6325 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 6495 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 2: 7405 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 7435 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 7486 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 5: 7484 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 7568 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 7: 8644 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 8671 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 8650 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 10: 8692 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 8685 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 12: 8716 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 13: 8712 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 8704 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 8721 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 8735 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 8749 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 18: 8746 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 8752 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 8744 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 8753 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 22: 8755 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 23: 8767 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 8764 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 8774 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 26: 8789 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 8769 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 28: 8790 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 8774 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 0: 7468 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 9283 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 2: 9418 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 9460 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 9491 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 5: 9542 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 9551 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 7: 9549 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 9597 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 9567 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 10: 9585 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 9619 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 12: 9613 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 13: 9625 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 9610 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 9630 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 9639 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 9627 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 18: 9628 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 9647 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 9671 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 9655 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 22: 9661 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 23: 9646 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 9653 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 9656 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 26: 9658 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 9660 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 28: 9643 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 9659 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 0: 9081 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 1: 9202 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 2: 9407 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 3: 9474 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 4: 9532 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 5: 9506 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 6: 9555 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 7: 9523 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 8: 9558 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 9: 9535 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 10: 9583 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 11: 9584 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 12: 9590 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 13: 9623 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 14: 9603 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 15: 9624 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 16: 9622 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 17: 9637 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 18: 9647 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 19: 9665 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 20: 9638 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 21: 9639 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 22: 9638 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 23: 9626 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 24: 9632 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 25: 9658 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 26: 9669 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 27: 9656 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 28: 9663 / 10000</t>
+  </si>
+  <si>
+    <t>Epoch 29: 9649 / 10000</t>
   </si>
 </sst>
 </file>
@@ -1067,6 +1752,18 @@
       <c r="H2" t="s">
         <v>186</v>
       </c>
+      <c r="I2" t="s">
+        <v>215</v>
+      </c>
+      <c r="J2" t="s">
+        <v>243</v>
+      </c>
+      <c r="K2" t="s">
+        <v>269</v>
+      </c>
+      <c r="L2" t="s">
+        <v>295</v>
+      </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3">
@@ -1090,6 +1787,18 @@
       <c r="H3" t="s">
         <v>187</v>
       </c>
+      <c r="I3" t="s">
+        <v>216</v>
+      </c>
+      <c r="J3" t="s">
+        <v>244</v>
+      </c>
+      <c r="K3" t="s">
+        <v>270</v>
+      </c>
+      <c r="L3" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4">
@@ -1113,6 +1822,18 @@
       <c r="H4" t="s">
         <v>188</v>
       </c>
+      <c r="I4" t="s">
+        <v>217</v>
+      </c>
+      <c r="J4" t="s">
+        <v>100</v>
+      </c>
+      <c r="K4" t="s">
+        <v>271</v>
+      </c>
+      <c r="L4" t="s">
+        <v>297</v>
+      </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5">
@@ -1136,6 +1857,18 @@
       <c r="H5" t="s">
         <v>189</v>
       </c>
+      <c r="I5" t="s">
+        <v>218</v>
+      </c>
+      <c r="J5" t="s">
+        <v>245</v>
+      </c>
+      <c r="K5" t="s">
+        <v>272</v>
+      </c>
+      <c r="L5" t="s">
+        <v>298</v>
+      </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -1159,6 +1892,18 @@
       <c r="H6" t="s">
         <v>190</v>
       </c>
+      <c r="I6" t="s">
+        <v>219</v>
+      </c>
+      <c r="J6" t="s">
+        <v>246</v>
+      </c>
+      <c r="K6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L6" t="s">
+        <v>299</v>
+      </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7">
@@ -1182,6 +1927,18 @@
       <c r="H7" t="s">
         <v>191</v>
       </c>
+      <c r="I7" t="s">
+        <v>220</v>
+      </c>
+      <c r="J7" t="s">
+        <v>247</v>
+      </c>
+      <c r="K7" t="s">
+        <v>131</v>
+      </c>
+      <c r="L7" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8">
@@ -1205,6 +1962,18 @@
       <c r="H8" t="s">
         <v>104</v>
       </c>
+      <c r="I8" t="s">
+        <v>221</v>
+      </c>
+      <c r="J8" t="s">
+        <v>248</v>
+      </c>
+      <c r="K8" t="s">
+        <v>274</v>
+      </c>
+      <c r="L8" t="s">
+        <v>300</v>
+      </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9">
@@ -1228,6 +1997,18 @@
       <c r="H9" t="s">
         <v>192</v>
       </c>
+      <c r="I9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J9" t="s">
+        <v>133</v>
+      </c>
+      <c r="K9" t="s">
+        <v>275</v>
+      </c>
+      <c r="L9" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10">
@@ -1251,6 +2032,18 @@
       <c r="H10" t="s">
         <v>193</v>
       </c>
+      <c r="I10" t="s">
+        <v>223</v>
+      </c>
+      <c r="J10" t="s">
+        <v>249</v>
+      </c>
+      <c r="K10" t="s">
+        <v>276</v>
+      </c>
+      <c r="L10" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11">
@@ -1274,6 +2067,18 @@
       <c r="H11" t="s">
         <v>194</v>
       </c>
+      <c r="I11" t="s">
+        <v>224</v>
+      </c>
+      <c r="J11" t="s">
+        <v>250</v>
+      </c>
+      <c r="K11" t="s">
+        <v>277</v>
+      </c>
+      <c r="L11" t="s">
+        <v>303</v>
+      </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12">
@@ -1297,6 +2102,18 @@
       <c r="H12" t="s">
         <v>195</v>
       </c>
+      <c r="I12" t="s">
+        <v>225</v>
+      </c>
+      <c r="J12" t="s">
+        <v>10</v>
+      </c>
+      <c r="K12" t="s">
+        <v>166</v>
+      </c>
+      <c r="L12" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13">
@@ -1320,6 +2137,18 @@
       <c r="H13" t="s">
         <v>196</v>
       </c>
+      <c r="I13" t="s">
+        <v>226</v>
+      </c>
+      <c r="J13" t="s">
+        <v>251</v>
+      </c>
+      <c r="K13" t="s">
+        <v>278</v>
+      </c>
+      <c r="L13" t="s">
+        <v>305</v>
+      </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14">
@@ -1343,6 +2172,18 @@
       <c r="H14" t="s">
         <v>197</v>
       </c>
+      <c r="I14" t="s">
+        <v>138</v>
+      </c>
+      <c r="J14" t="s">
+        <v>252</v>
+      </c>
+      <c r="K14" t="s">
+        <v>279</v>
+      </c>
+      <c r="L14" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15">
@@ -1366,6 +2207,18 @@
       <c r="H15" t="s">
         <v>198</v>
       </c>
+      <c r="I15" t="s">
+        <v>227</v>
+      </c>
+      <c r="J15" t="s">
+        <v>253</v>
+      </c>
+      <c r="K15" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -1389,8 +2242,20 @@
       <c r="H16" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I16" t="s">
+        <v>228</v>
+      </c>
+      <c r="J16" t="s">
+        <v>254</v>
+      </c>
+      <c r="K16" t="s">
+        <v>280</v>
+      </c>
+      <c r="L16" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>15</v>
       </c>
@@ -1412,8 +2277,20 @@
       <c r="H17" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I17" t="s">
+        <v>229</v>
+      </c>
+      <c r="J17" t="s">
+        <v>255</v>
+      </c>
+      <c r="K17" t="s">
+        <v>281</v>
+      </c>
+      <c r="L17" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>16</v>
       </c>
@@ -1435,8 +2312,20 @@
       <c r="H18" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I18" t="s">
+        <v>230</v>
+      </c>
+      <c r="J18" t="s">
+        <v>256</v>
+      </c>
+      <c r="K18" t="s">
+        <v>282</v>
+      </c>
+      <c r="L18" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>17</v>
       </c>
@@ -1458,8 +2347,20 @@
       <c r="H19" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I19" t="s">
+        <v>231</v>
+      </c>
+      <c r="J19" t="s">
+        <v>257</v>
+      </c>
+      <c r="K19" t="s">
+        <v>283</v>
+      </c>
+      <c r="L19" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>18</v>
       </c>
@@ -1481,8 +2382,20 @@
       <c r="H20" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I20" t="s">
+        <v>232</v>
+      </c>
+      <c r="J20" t="s">
+        <v>258</v>
+      </c>
+      <c r="K20" t="s">
+        <v>284</v>
+      </c>
+      <c r="L20" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>19</v>
       </c>
@@ -1504,8 +2417,20 @@
       <c r="H21" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I21" t="s">
+        <v>233</v>
+      </c>
+      <c r="J21" t="s">
+        <v>259</v>
+      </c>
+      <c r="K21" t="s">
+        <v>285</v>
+      </c>
+      <c r="L21" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>20</v>
       </c>
@@ -1527,8 +2452,20 @@
       <c r="H22" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I22" t="s">
+        <v>234</v>
+      </c>
+      <c r="J22" t="s">
+        <v>260</v>
+      </c>
+      <c r="K22" t="s">
+        <v>286</v>
+      </c>
+      <c r="L22" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>21</v>
       </c>
@@ -1550,8 +2487,20 @@
       <c r="H23" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I23" t="s">
+        <v>235</v>
+      </c>
+      <c r="J23" t="s">
+        <v>261</v>
+      </c>
+      <c r="K23" t="s">
+        <v>287</v>
+      </c>
+      <c r="L23" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>22</v>
       </c>
@@ -1573,8 +2522,20 @@
       <c r="H24" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I24" t="s">
+        <v>148</v>
+      </c>
+      <c r="J24" t="s">
+        <v>262</v>
+      </c>
+      <c r="K24" t="s">
+        <v>288</v>
+      </c>
+      <c r="L24" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>23</v>
       </c>
@@ -1596,8 +2557,20 @@
       <c r="H25" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I25" t="s">
+        <v>236</v>
+      </c>
+      <c r="J25" t="s">
+        <v>263</v>
+      </c>
+      <c r="K25" t="s">
+        <v>23</v>
+      </c>
+      <c r="L25" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>24</v>
       </c>
@@ -1619,8 +2592,20 @@
       <c r="H26" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I26" t="s">
+        <v>237</v>
+      </c>
+      <c r="J26" t="s">
+        <v>264</v>
+      </c>
+      <c r="K26" t="s">
+        <v>289</v>
+      </c>
+      <c r="L26" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>25</v>
       </c>
@@ -1642,8 +2627,20 @@
       <c r="H27" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I27" t="s">
+        <v>238</v>
+      </c>
+      <c r="J27" t="s">
+        <v>265</v>
+      </c>
+      <c r="K27" t="s">
+        <v>290</v>
+      </c>
+      <c r="L27" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>26</v>
       </c>
@@ -1665,8 +2662,20 @@
       <c r="H28" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I28" t="s">
+        <v>239</v>
+      </c>
+      <c r="J28" t="s">
+        <v>266</v>
+      </c>
+      <c r="K28" t="s">
+        <v>291</v>
+      </c>
+      <c r="L28" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29">
         <v>27</v>
       </c>
@@ -1688,8 +2697,20 @@
       <c r="H29" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I29" t="s">
+        <v>240</v>
+      </c>
+      <c r="J29" t="s">
+        <v>267</v>
+      </c>
+      <c r="K29" t="s">
+        <v>292</v>
+      </c>
+      <c r="L29" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30">
         <v>28</v>
       </c>
@@ -1711,8 +2732,20 @@
       <c r="H30" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I30" t="s">
+        <v>241</v>
+      </c>
+      <c r="J30" t="s">
+        <v>183</v>
+      </c>
+      <c r="K30" t="s">
+        <v>293</v>
+      </c>
+      <c r="L30" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31">
         <v>29</v>
       </c>
@@ -1733,6 +2766,18 @@
       </c>
       <c r="H31" t="s">
         <v>214</v>
+      </c>
+      <c r="I31" t="s">
+        <v>242</v>
+      </c>
+      <c r="J31" t="s">
+        <v>268</v>
+      </c>
+      <c r="K31" t="s">
+        <v>294</v>
+      </c>
+      <c r="L31" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.25">
@@ -1883,6 +2928,557 @@
     <row r="62" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D62" t="s">
         <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B609DA57-4304-46EB-8B8F-CE3F33BB4214}">
+  <dimension ref="C1:H32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="5" width="25.7109375" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="9" width="25.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>351</v>
+      </c>
+      <c r="G1" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="2" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>321</v>
+      </c>
+      <c r="E3" t="s">
+        <v>353</v>
+      </c>
+      <c r="G3" t="s">
+        <v>383</v>
+      </c>
+      <c r="H3" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="4" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>322</v>
+      </c>
+      <c r="E4" t="s">
+        <v>354</v>
+      </c>
+      <c r="G4" t="s">
+        <v>384</v>
+      </c>
+      <c r="H4" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="5" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>323</v>
+      </c>
+      <c r="E5" t="s">
+        <v>355</v>
+      </c>
+      <c r="G5" t="s">
+        <v>385</v>
+      </c>
+      <c r="H5" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="6" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>324</v>
+      </c>
+      <c r="E6" t="s">
+        <v>356</v>
+      </c>
+      <c r="G6" t="s">
+        <v>386</v>
+      </c>
+      <c r="H6" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="7" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>325</v>
+      </c>
+      <c r="E7" t="s">
+        <v>357</v>
+      </c>
+      <c r="G7" t="s">
+        <v>387</v>
+      </c>
+      <c r="H7" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="8" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E8" t="s">
+        <v>358</v>
+      </c>
+      <c r="G8" t="s">
+        <v>388</v>
+      </c>
+      <c r="H8" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="9" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>327</v>
+      </c>
+      <c r="E9" t="s">
+        <v>359</v>
+      </c>
+      <c r="G9" t="s">
+        <v>389</v>
+      </c>
+      <c r="H9" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="10" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>328</v>
+      </c>
+      <c r="E10" t="s">
+        <v>360</v>
+      </c>
+      <c r="G10" t="s">
+        <v>390</v>
+      </c>
+      <c r="H10" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="11" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C11">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>329</v>
+      </c>
+      <c r="E11" t="s">
+        <v>361</v>
+      </c>
+      <c r="G11" t="s">
+        <v>391</v>
+      </c>
+      <c r="H11" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="12" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C12">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>330</v>
+      </c>
+      <c r="E12" t="s">
+        <v>362</v>
+      </c>
+      <c r="G12" t="s">
+        <v>392</v>
+      </c>
+      <c r="H12" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="13" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C13">
+        <v>10</v>
+      </c>
+      <c r="D13" t="s">
+        <v>331</v>
+      </c>
+      <c r="E13" t="s">
+        <v>363</v>
+      </c>
+      <c r="G13" t="s">
+        <v>393</v>
+      </c>
+      <c r="H13" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="14" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C14">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>332</v>
+      </c>
+      <c r="E14" t="s">
+        <v>364</v>
+      </c>
+      <c r="G14" t="s">
+        <v>394</v>
+      </c>
+      <c r="H14" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="15" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <v>12</v>
+      </c>
+      <c r="D15" t="s">
+        <v>333</v>
+      </c>
+      <c r="E15" t="s">
+        <v>365</v>
+      </c>
+      <c r="G15" t="s">
+        <v>395</v>
+      </c>
+      <c r="H15" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="16" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>334</v>
+      </c>
+      <c r="E16" t="s">
+        <v>366</v>
+      </c>
+      <c r="G16" t="s">
+        <v>396</v>
+      </c>
+      <c r="H16" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>14</v>
+      </c>
+      <c r="D17" t="s">
+        <v>335</v>
+      </c>
+      <c r="E17" t="s">
+        <v>367</v>
+      </c>
+      <c r="G17" t="s">
+        <v>397</v>
+      </c>
+      <c r="H17" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>336</v>
+      </c>
+      <c r="E18" t="s">
+        <v>368</v>
+      </c>
+      <c r="G18" t="s">
+        <v>398</v>
+      </c>
+      <c r="H18" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>337</v>
+      </c>
+      <c r="E19" t="s">
+        <v>369</v>
+      </c>
+      <c r="G19" t="s">
+        <v>399</v>
+      </c>
+      <c r="H19" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>17</v>
+      </c>
+      <c r="D20" t="s">
+        <v>338</v>
+      </c>
+      <c r="E20" t="s">
+        <v>370</v>
+      </c>
+      <c r="G20" t="s">
+        <v>400</v>
+      </c>
+      <c r="H20" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <v>18</v>
+      </c>
+      <c r="D21" t="s">
+        <v>339</v>
+      </c>
+      <c r="E21" t="s">
+        <v>371</v>
+      </c>
+      <c r="G21" t="s">
+        <v>401</v>
+      </c>
+      <c r="H21" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="22" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C22">
+        <v>19</v>
+      </c>
+      <c r="D22" t="s">
+        <v>340</v>
+      </c>
+      <c r="E22" t="s">
+        <v>372</v>
+      </c>
+      <c r="G22" t="s">
+        <v>402</v>
+      </c>
+      <c r="H22" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="23" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C23">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
+        <v>341</v>
+      </c>
+      <c r="E23" t="s">
+        <v>373</v>
+      </c>
+      <c r="G23" t="s">
+        <v>403</v>
+      </c>
+      <c r="H23" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C24">
+        <v>21</v>
+      </c>
+      <c r="D24" t="s">
+        <v>342</v>
+      </c>
+      <c r="E24" t="s">
+        <v>374</v>
+      </c>
+      <c r="G24" t="s">
+        <v>404</v>
+      </c>
+      <c r="H24" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C25">
+        <v>22</v>
+      </c>
+      <c r="D25" t="s">
+        <v>343</v>
+      </c>
+      <c r="E25" t="s">
+        <v>375</v>
+      </c>
+      <c r="G25" t="s">
+        <v>405</v>
+      </c>
+      <c r="H25" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="26" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C26">
+        <v>23</v>
+      </c>
+      <c r="D26" t="s">
+        <v>344</v>
+      </c>
+      <c r="E26" t="s">
+        <v>376</v>
+      </c>
+      <c r="G26" t="s">
+        <v>406</v>
+      </c>
+      <c r="H26" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C27">
+        <v>24</v>
+      </c>
+      <c r="D27" t="s">
+        <v>345</v>
+      </c>
+      <c r="E27" t="s">
+        <v>377</v>
+      </c>
+      <c r="G27" t="s">
+        <v>407</v>
+      </c>
+      <c r="H27" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="28" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C28">
+        <v>25</v>
+      </c>
+      <c r="D28" t="s">
+        <v>346</v>
+      </c>
+      <c r="E28" t="s">
+        <v>378</v>
+      </c>
+      <c r="G28" t="s">
+        <v>408</v>
+      </c>
+      <c r="H28" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="29" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C29">
+        <v>26</v>
+      </c>
+      <c r="D29" t="s">
+        <v>347</v>
+      </c>
+      <c r="E29" t="s">
+        <v>379</v>
+      </c>
+      <c r="G29" t="s">
+        <v>409</v>
+      </c>
+      <c r="H29" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="30" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C30">
+        <v>27</v>
+      </c>
+      <c r="D30" t="s">
+        <v>348</v>
+      </c>
+      <c r="E30" t="s">
+        <v>380</v>
+      </c>
+      <c r="G30" t="s">
+        <v>410</v>
+      </c>
+      <c r="H30" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="31" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C31">
+        <v>28</v>
+      </c>
+      <c r="D31" t="s">
+        <v>349</v>
+      </c>
+      <c r="E31" t="s">
+        <v>381</v>
+      </c>
+      <c r="G31" t="s">
+        <v>411</v>
+      </c>
+      <c r="H31" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="32" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C32">
+        <v>29</v>
+      </c>
+      <c r="D32" t="s">
+        <v>350</v>
+      </c>
+      <c r="E32" t="s">
+        <v>382</v>
+      </c>
+      <c r="G32" t="s">
+        <v>412</v>
+      </c>
+      <c r="H32" t="s">
+        <v>442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>